<commit_message>
Add full inference testbench and update simulation files
</commit_message>
<xml_diff>
--- a/Milestone Tracker.xlsx
+++ b/Milestone Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liche/finn/Design-Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E53BC1C0-43A2-4144-8C76-DAB511D04A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F01BCA3-A444-B042-A9B9-2FCC2D95F248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,9 +36,6 @@
     <t>Project Name</t>
   </si>
   <si>
-    <t>Tiny CNN CIFAR-10 Accelerator on Basys 3 FPGA</t>
-  </si>
-  <si>
     <t>Legend</t>
   </si>
   <si>
@@ -193,6 +190,9 @@
   </si>
   <si>
     <t xml:space="preserve"> review: FPGA CNN accelerators</t>
+  </si>
+  <si>
+    <t>CNN CIFAR-10 Accelerator on Basys 3 FPGA</t>
   </si>
 </sst>
 </file>
@@ -1601,17 +1601,17 @@
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="72" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>6</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>7</v>
       </c>
       <c r="H4" s="10"/>
       <c r="I4" s="2"/>
@@ -1630,18 +1630,18 @@
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2"/>
       <c r="B5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>8</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>9</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="73"/>
       <c r="F5" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>10</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>11</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="2"/>
@@ -1660,18 +1660,18 @@
     <row r="6" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>13</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="74"/>
       <c r="F6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="15" t="s">
         <v>14</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>15</v>
       </c>
       <c r="H6" s="16"/>
       <c r="I6" s="2"/>
@@ -1715,28 +1715,28 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="68" t="s">
         <v>16</v>
-      </c>
-      <c r="F8" s="68" t="s">
-        <v>17</v>
       </c>
       <c r="G8" s="69"/>
       <c r="H8" s="70"/>
       <c r="I8" s="71" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J8" s="69"/>
       <c r="K8" s="69"/>
       <c r="L8" s="70"/>
       <c r="M8" s="68" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="N8" s="69"/>
       <c r="O8" s="69"/>
       <c r="P8" s="69"/>
       <c r="Q8" s="70"/>
       <c r="R8" s="75" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="S8" s="76"/>
       <c r="T8" s="2"/>
@@ -1747,7 +1747,7 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F9" s="19">
         <v>11</v>
@@ -1799,7 +1799,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F10" s="27">
         <v>1</v>
@@ -1848,16 +1848,16 @@
     <row r="11" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2"/>
       <c r="B11" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="D11" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="E11" s="36" t="s">
         <v>25</v>
-      </c>
-      <c r="E11" s="36" t="s">
-        <v>26</v>
       </c>
       <c r="F11" s="37"/>
       <c r="G11" s="37"/>
@@ -1878,19 +1878,19 @@
     <row r="12" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="2"/>
       <c r="B12" s="62" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="39" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="39" t="s">
+      <c r="E12" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="40" t="s">
-        <v>29</v>
-      </c>
       <c r="F12" s="41" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G12" s="42"/>
       <c r="H12" s="43"/>
@@ -1910,19 +1910,19 @@
     <row r="13" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2"/>
       <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="46" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="46" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="47" t="s">
-        <v>28</v>
-      </c>
       <c r="F13" s="41" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G13" s="41"/>
       <c r="H13" s="48"/>
@@ -1942,22 +1942,22 @@
     <row r="14" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2"/>
       <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="46" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="46" t="s">
+      <c r="E14" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="47" t="s">
-        <v>29</v>
-      </c>
       <c r="F14" s="41" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G14" s="49" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H14" s="41"/>
       <c r="I14" s="41"/>
@@ -1976,23 +1976,23 @@
     <row r="15" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2"/>
       <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="46" t="s">
-        <v>33</v>
-      </c>
       <c r="D15" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="47" t="s">
         <v>28</v>
-      </c>
-      <c r="E15" s="47" t="s">
-        <v>29</v>
       </c>
       <c r="F15" s="51"/>
       <c r="G15" s="52" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H15" s="53" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I15" s="41"/>
       <c r="J15" s="52"/>
@@ -2010,24 +2010,24 @@
     <row r="16" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2"/>
       <c r="B16" s="63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" s="46" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D16" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="47" t="s">
         <v>28</v>
-      </c>
-      <c r="E16" s="47" t="s">
-        <v>29</v>
       </c>
       <c r="F16" s="44"/>
       <c r="G16" s="42"/>
       <c r="H16" s="43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I16" s="44" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J16" s="41"/>
       <c r="K16" s="42"/>
@@ -2044,22 +2044,22 @@
     <row r="17" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2"/>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C17" s="46" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D17" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="47" t="s">
         <v>28</v>
-      </c>
-      <c r="E17" s="47" t="s">
-        <v>29</v>
       </c>
       <c r="F17" s="41"/>
       <c r="G17" s="49"/>
       <c r="H17" s="48"/>
       <c r="I17" s="41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J17" s="49"/>
       <c r="K17" s="41"/>
@@ -2076,25 +2076,25 @@
     <row r="18" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2"/>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D18" s="46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E18" s="47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F18" s="41"/>
       <c r="G18" s="49"/>
       <c r="H18" s="48"/>
       <c r="I18" s="41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J18" s="49" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K18" s="49"/>
       <c r="L18" s="41"/>
@@ -2110,26 +2110,26 @@
     <row r="19" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="2"/>
       <c r="B19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="46" t="s">
-        <v>38</v>
-      </c>
       <c r="D19" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="47" t="s">
         <v>28</v>
-      </c>
-      <c r="E19" s="47" t="s">
-        <v>29</v>
       </c>
       <c r="F19" s="51"/>
       <c r="G19" s="52"/>
       <c r="H19" s="53"/>
       <c r="I19" s="51"/>
       <c r="J19" s="52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K19" s="52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L19" s="53"/>
       <c r="M19" s="41"/>
@@ -2144,16 +2144,16 @@
     <row r="20" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2"/>
       <c r="B20" s="63" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="46" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D20" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="47" t="s">
         <v>28</v>
-      </c>
-      <c r="E20" s="47" t="s">
-        <v>29</v>
       </c>
       <c r="F20" s="44"/>
       <c r="G20" s="42"/>
@@ -2161,7 +2161,7 @@
       <c r="I20" s="44"/>
       <c r="J20" s="42"/>
       <c r="K20" s="42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="44"/>
@@ -2176,16 +2176,16 @@
     <row r="21" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="2"/>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C21" s="46" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D21" s="46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E21" s="47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F21" s="41"/>
       <c r="G21" s="49"/>
@@ -2193,10 +2193,10 @@
       <c r="I21" s="41"/>
       <c r="J21" s="49"/>
       <c r="K21" s="49" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L21" s="48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M21" s="41"/>
       <c r="N21" s="49"/>
@@ -2210,16 +2210,16 @@
     <row r="22" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2"/>
       <c r="B22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="46" t="s">
-        <v>42</v>
-      </c>
       <c r="D22" s="46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E22" s="47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F22" s="51"/>
       <c r="G22" s="52"/>
@@ -2227,13 +2227,13 @@
       <c r="I22" s="51"/>
       <c r="J22" s="52"/>
       <c r="K22" s="52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L22" s="53" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M22" s="51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N22" s="52"/>
       <c r="O22" s="52"/>
@@ -2246,16 +2246,16 @@
     <row r="23" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="2"/>
       <c r="B23" s="55" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" s="56" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D23" s="56" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E23" s="57" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F23" s="58"/>
       <c r="G23" s="59"/>
@@ -2264,13 +2264,13 @@
       <c r="J23" s="59"/>
       <c r="K23" s="59"/>
       <c r="L23" s="60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M23" s="58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N23" s="59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O23" s="59"/>
       <c r="P23" s="59"/>
@@ -2282,16 +2282,16 @@
     <row r="24" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -2301,10 +2301,10 @@
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
       <c r="M24" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
@@ -2315,176 +2315,176 @@
     </row>
     <row r="25" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" t="s">
         <v>47</v>
       </c>
-      <c r="C27" t="s">
-        <v>48</v>
-      </c>
       <c r="D27" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" t="s">
         <v>28</v>
       </c>
-      <c r="E27" t="s">
-        <v>29</v>
-      </c>
       <c r="M27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" t="s">
         <v>28</v>
       </c>
-      <c r="E28" t="s">
-        <v>29</v>
-      </c>
       <c r="N28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B29" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C29" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" t="s">
         <v>28</v>
       </c>
-      <c r="E29" t="s">
-        <v>29</v>
-      </c>
       <c r="P29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B30" t="s">
+        <v>50</v>
+      </c>
+      <c r="C30" t="s">
         <v>51</v>
       </c>
-      <c r="C30" t="s">
-        <v>52</v>
-      </c>
       <c r="D30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Q30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B32" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E32" t="s">
         <v>28</v>
       </c>
-      <c r="E32" t="s">
-        <v>29</v>
-      </c>
       <c r="R32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C33" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E33" t="s">
         <v>28</v>
       </c>
-      <c r="E33" t="s">
-        <v>29</v>
-      </c>
       <c r="S33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>